<commit_message>
Updated project files and cleaned repository
</commit_message>
<xml_diff>
--- a/input/employees.xlsx
+++ b/input/employees.xlsx
@@ -27,9 +27,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
-    <t>Page</t>
+    <t>Matricule</t>
   </si>
   <si>
     <t>Name</t>
@@ -45,12 +45,6 @@
   </si>
   <si>
     <t>Mary</t>
-  </si>
-  <si>
-    <t>ebakovo@gmail.com</t>
-  </si>
-  <si>
-    <t>Joy</t>
   </si>
   <si>
     <t>nerisbi801@gmail.com</t>
@@ -669,11 +663,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1212,6 +1209,8 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3" outlineLevelCol="2"/>
   <cols>
+    <col min="1" max="1" width="18.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="16.7142857142857" customWidth="1"/>
     <col min="3" max="3" width="21.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1228,7 +1227,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2">
-        <v>1</v>
+        <v>3060</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1239,31 +1238,22 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>8</v>
-      </c>
+    <row r="4" spans="3:3">
+      <c r="C4" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" display="ebakop@crtv.cm" tooltip="mailto:ebakop@crtv.cm"/>
-    <hyperlink ref="C3" r:id="rId2" display="ebakovo@gmail.com" tooltip="mailto:ebakovo@gmail.com"/>
-    <hyperlink ref="C4" r:id="rId3" display="nerisbi801@gmail.com" tooltip="mailto:nerisbi801@gmail.com"/>
+    <hyperlink ref="C3" r:id="rId2" display="nerisbi801@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Revert "Updated project files and cleaned repository"
This reverts commit d4acbbe4c41ec9841c4f25ad76d53b756d55310b.
</commit_message>
<xml_diff>
--- a/input/employees.xlsx
+++ b/input/employees.xlsx
@@ -27,9 +27,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
-    <t>Matricule</t>
+    <t>Page</t>
   </si>
   <si>
     <t>Name</t>
@@ -45,6 +45,12 @@
   </si>
   <si>
     <t>Mary</t>
+  </si>
+  <si>
+    <t>ebakovo@gmail.com</t>
+  </si>
+  <si>
+    <t>Joy</t>
   </si>
   <si>
     <t>nerisbi801@gmail.com</t>
@@ -663,14 +669,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1209,8 +1212,6 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="18.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="16.7142857142857" customWidth="1"/>
     <col min="3" max="3" width="21.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1227,7 +1228,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2">
-        <v>3060</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1238,22 +1239,31 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="3:3">
-      <c r="C4" s="1"/>
+    <row r="4" spans="1:3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" display="ebakop@crtv.cm" tooltip="mailto:ebakop@crtv.cm"/>
-    <hyperlink ref="C3" r:id="rId2" display="nerisbi801@gmail.com"/>
+    <hyperlink ref="C3" r:id="rId2" display="ebakovo@gmail.com" tooltip="mailto:ebakovo@gmail.com"/>
+    <hyperlink ref="C4" r:id="rId3" display="nerisbi801@gmail.com" tooltip="mailto:nerisbi801@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>